<commit_message>
Atualização no projeto em Excel da UC3
</commit_message>
<xml_diff>
--- a/UC3/Exercicios/EX002/Pet shop ex02-uc3.xlsx
+++ b/UC3/Exercicios/EX002/Pet shop ex02-uc3.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabri\OneDrive\Documentos\estudos-prog\estudos\TDS-Senac\UC3\Exercicios\EX002\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B987012-DAD2-4B63-B0C6-35BF63D05CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62DA8C57-2E19-44EF-ACE4-B804DE81F678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A77BCF53-0E97-4906-BD97-7490673142B7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A77BCF53-0E97-4906-BD97-7490673142B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Requisitos Funcionais" sheetId="1" r:id="rId1"/>
     <sheet name="Possíveis Tabelas" sheetId="2" r:id="rId2"/>
     <sheet name="Dicionário de Dados" sheetId="3" r:id="rId3"/>
+    <sheet name="Clientes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,8 +41,27 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={66327E8A-759F-42CA-8E79-36683DF49B7D}</author>
+  </authors>
+  <commentList>
+    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{66327E8A-759F-42CA-8E79-36683DF49B7D}">
+      <text>
+        <t xml:space="preserve">[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Era pra ser 5551912345678, mas ele traduz para cálculos que usam E.
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="65">
   <si>
     <t xml:space="preserve">1. </t>
   </si>
@@ -109,18 +129,6 @@
     <t>Serviços realizados, datas, valores</t>
   </si>
   <si>
-    <t>Agenda</t>
-  </si>
-  <si>
-    <t>Animais cadastrados para atendimento: valor, hora, serviços</t>
-  </si>
-  <si>
-    <t>Histórico</t>
-  </si>
-  <si>
-    <t>Animais onde serviços já foram realizados: valor, hora, serviços</t>
-  </si>
-  <si>
     <t>Campo</t>
   </si>
   <si>
@@ -163,17 +171,98 @@
     <t>animal_id</t>
   </si>
   <si>
-    <t>ID do animal (até 99,999)</t>
-  </si>
-  <si>
-    <t>Nome do animal (por quê não?)</t>
+    <t>breed</t>
+  </si>
+  <si>
+    <t>Raça do animal</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>Número de telefone para contato</t>
+  </si>
+  <si>
+    <t>cpf</t>
+  </si>
+  <si>
+    <t>CPF do cliente</t>
+  </si>
+  <si>
+    <t>Data/Hora</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Horário do atendimento</t>
+  </si>
+  <si>
+    <t>Identificador do atendimento</t>
+  </si>
+  <si>
+    <t>service_id</t>
+  </si>
+  <si>
+    <t>Identificador do cliente (Clientes)</t>
+  </si>
+  <si>
+    <t>Identificador do animal (Animais)</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Decimal</t>
+  </si>
+  <si>
+    <t>Valor do atendimento</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Status do atendimento ("Concluído", "Agendado" ou "Cancelado")</t>
+  </si>
+  <si>
+    <t>Identificador do animal</t>
+  </si>
+  <si>
+    <t>Nome do animal</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>Peso do animal</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
+    <t>Serviço que será realizado</t>
+  </si>
+  <si>
+    <t>J.R.R. Tolkien</t>
+  </si>
+  <si>
+    <t>callMeLord@gmail.com</t>
+  </si>
+  <si>
+    <t>YouShallNotPass1954</t>
+  </si>
+  <si>
+    <t>010.202.393-45</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,6 +301,20 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -236,8 +339,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -249,11 +353,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -265,8 +368,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -280,6 +387,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="VALDIR GABRIEL PINHEIRO DE LARA" id="{6BDBFB2D-430A-431B-B0AF-2CFB9C3FB8EC}" userId="S::04503720066@senacrs.edu.br::34f2291b-7fcb-4070-8dd1-3f6dda9bd691" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -597,6 +710,15 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="E2" dT="2026-07-28T02:20:10.56" personId="{6BDBFB2D-430A-431B-B0AF-2CFB9C3FB8EC}" id="{66327E8A-759F-42CA-8E79-36683DF49B7D}">
+    <text xml:space="preserve">Era pra ser 5551912345678, mas ele traduz para cálculos que usam E.
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0572D44-E8C8-4BC5-B3BE-2B79D7A1CB63}">
   <dimension ref="A1:B16"/>
@@ -615,50 +737,50 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -691,7 +813,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
@@ -699,7 +821,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B3" t="s">
@@ -707,7 +829,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
@@ -715,20 +837,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -770,12 +879,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C4987F1-C2F1-4B23-BBE4-D33E26D37EC7}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="34.28515625" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="61.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -783,148 +893,482 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="8">
+        <v>5</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="7">
+        <v>100</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="8">
+        <v>254</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="9" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="8">
+        <v>18</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="9">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="8">
+        <v>13</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="8">
+        <v>11</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="8">
         <v>5</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E8" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="8">
+        <v>5</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="C10" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="8">
+        <v>100</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="8">
-        <v>100</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="C11" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="8">
+        <v>42</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="9">
-        <v>254</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="D13" s="8">
+        <v>11</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="8">
+        <v>5</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="9">
-        <v>18</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="C15" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="8">
+        <v>5</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="8">
+        <v>256</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="8">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="8">
+        <v>25</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="9">
-        <v>5</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="9">
-        <v>100</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+      <c r="C19" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="9"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="E30" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3792A4EE-4C0A-4385-A5BD-9790C0B3D0D2}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="8">
+        <v>5551912345678</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{E4A45386-2BC1-453F-8D40-FEB05638A3E1}"/>
+  </hyperlinks>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>